<commit_message>
Avaliação manual os 25 primeiros registros - Filipe
</commit_message>
<xml_diff>
--- a/avaliacao/Filipe/ouro_Filipe.xlsx
+++ b/avaliacao/Filipe/ouro_Filipe.xlsx
@@ -4,19 +4,19 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="sobre" sheetId="1" r:id="rId1"/>
     <sheet name="leis" sheetId="2" r:id="rId2"/>
     <sheet name="ouro" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8740" uniqueCount="1923">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8768" uniqueCount="1929">
   <si>
     <t>campo</t>
   </si>
@@ -5785,6 +5785,24 @@
   </si>
   <si>
     <t>Claude</t>
+  </si>
+  <si>
+    <t>Filipe</t>
+  </si>
+  <si>
+    <t>Manter</t>
+  </si>
+  <si>
+    <t>Corrigir</t>
+  </si>
+  <si>
+    <t>O parágrafo § 1º estava unido ao texto do artigo Art. 2º. Foi necessário separar.</t>
+  </si>
+  <si>
+    <t>Sem ementa</t>
+  </si>
+  <si>
+    <t>O artigo 10, inciso I estava com o inciso II unido no texto, sendo que era apenas uma referência no texto para indicar o inciso II.</t>
   </si>
 </sst>
 </file>
@@ -5807,12 +5825,24 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -5831,9 +5861,14 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5845,9 +5880,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Escritório">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5885,7 +5920,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Escritório">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -5955,7 +5990,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Escritório">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -6131,6 +6166,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -6189,6 +6228,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I126"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="4" max="4" width="112.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="7" max="7" width="217" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
@@ -6220,544 +6268,642 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>1936</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I2" t="s">
-        <v>402</v>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>1937</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" s="3">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>1926</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1935</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" s="3">
+        <v>4</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1937</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="E5" s="3">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1937</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="E6" s="3">
+        <v>2</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1951</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="E7" s="2">
+        <v>25</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I3" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4">
-        <v>1935</v>
-      </c>
-      <c r="C4" t="s">
-        <v>147</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="E4">
-        <v>4</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G7" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1955</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E8" s="2">
+        <v>9</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I4" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5">
-        <v>1937</v>
-      </c>
-      <c r="C5" t="s">
-        <v>148</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G8" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1957</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="E9" s="2">
+        <v>21</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1964</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="E10" s="2">
+        <v>52</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1966</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E11" s="2">
+        <v>45</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I5" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6">
-        <v>1937</v>
-      </c>
-      <c r="C6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G11" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1968</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="E12" s="2">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I6" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7">
-        <v>1951</v>
-      </c>
-      <c r="C7" t="s">
-        <v>150</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="E7">
-        <v>25</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="2">
+        <v>1971</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="E13" s="2">
+        <v>7</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="G7" t="s">
-        <v>397</v>
-      </c>
-      <c r="I7" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8">
-        <v>1955</v>
-      </c>
-      <c r="C8" t="s">
-        <v>151</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="E8">
-        <v>9</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="2">
+        <v>1973</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" s="2">
+        <v>44</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="G8" t="s">
-        <v>398</v>
-      </c>
-      <c r="I8" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9">
-        <v>1957</v>
-      </c>
-      <c r="C9" t="s">
-        <v>152</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="E9">
-        <v>21</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="2">
+        <v>1948</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="E15" s="2">
+        <v>6</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="2">
+        <v>1975</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="E16" s="2">
+        <v>13</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="2">
+        <v>1977</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="E17" s="2">
+        <v>8</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="2">
+        <v>1979</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="E18" s="2">
+        <v>7</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="2">
+        <v>1981</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="E19" s="2">
+        <v>7</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="2">
+        <v>1981</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E20" s="2">
+        <v>13</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="G9" t="s">
-        <v>399</v>
-      </c>
-      <c r="I9" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10">
-        <v>1964</v>
-      </c>
-      <c r="C10" t="s">
-        <v>153</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="E10">
-        <v>52</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G20" s="2"/>
+      <c r="H20" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="2">
+        <v>1984</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="E21" s="2">
+        <v>6</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="2">
+        <v>1985</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="E22" s="2">
+        <v>8</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="I10" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11">
-        <v>1966</v>
-      </c>
-      <c r="C11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="E11">
-        <v>45</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G22" s="2"/>
+      <c r="H22" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="3">
+        <v>1986</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="E23" s="3">
+        <v>57</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>1928</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="2">
+        <v>1987</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="E24" s="2">
+        <v>6</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="G11" t="s">
-        <v>400</v>
-      </c>
-      <c r="I11" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12">
-        <v>1968</v>
-      </c>
-      <c r="C12" t="s">
-        <v>155</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="E12">
-        <v>10</v>
-      </c>
-      <c r="F12" t="s">
-        <v>395</v>
-      </c>
-      <c r="I12" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13">
-        <v>1971</v>
-      </c>
-      <c r="C13" t="s">
-        <v>156</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="E13">
-        <v>7</v>
-      </c>
-      <c r="F13" t="s">
-        <v>395</v>
-      </c>
-      <c r="I13" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14">
-        <v>1973</v>
-      </c>
-      <c r="C14" t="s">
-        <v>157</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="E14">
-        <v>44</v>
-      </c>
-      <c r="F14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I14" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15">
-        <v>1948</v>
-      </c>
-      <c r="C15" t="s">
-        <v>158</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="E15">
-        <v>6</v>
-      </c>
-      <c r="F15" t="s">
-        <v>395</v>
-      </c>
-      <c r="I15" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16">
-        <v>1975</v>
-      </c>
-      <c r="C16" t="s">
-        <v>159</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="E16">
-        <v>13</v>
-      </c>
-      <c r="F16" t="s">
-        <v>395</v>
-      </c>
-      <c r="I16" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17">
-        <v>1977</v>
-      </c>
-      <c r="C17" t="s">
-        <v>160</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="E17">
-        <v>8</v>
-      </c>
-      <c r="F17" t="s">
-        <v>395</v>
-      </c>
-      <c r="I17" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18">
-        <v>1979</v>
-      </c>
-      <c r="C18" t="s">
-        <v>161</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="E18">
-        <v>7</v>
-      </c>
-      <c r="F18" t="s">
-        <v>395</v>
-      </c>
-      <c r="I18" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19">
-        <v>1981</v>
-      </c>
-      <c r="C19" t="s">
-        <v>162</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="E19">
-        <v>7</v>
-      </c>
-      <c r="F19" t="s">
-        <v>395</v>
-      </c>
-      <c r="I19" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20">
-        <v>1981</v>
-      </c>
-      <c r="C20" t="s">
-        <v>163</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="E20">
-        <v>13</v>
-      </c>
-      <c r="F20" t="s">
-        <v>396</v>
-      </c>
-      <c r="I20" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B21">
-        <v>1984</v>
-      </c>
-      <c r="C21" t="s">
-        <v>164</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="E21">
-        <v>6</v>
-      </c>
-      <c r="F21" t="s">
-        <v>395</v>
-      </c>
-      <c r="I21" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22">
-        <v>1985</v>
-      </c>
-      <c r="C22" t="s">
-        <v>165</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="E22">
-        <v>8</v>
-      </c>
-      <c r="F22" t="s">
-        <v>396</v>
-      </c>
-      <c r="I22" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23">
-        <v>1986</v>
-      </c>
-      <c r="C23" t="s">
-        <v>166</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="E23">
-        <v>58</v>
-      </c>
-      <c r="F23" t="s">
-        <v>396</v>
-      </c>
-      <c r="I23" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24">
-        <v>1987</v>
-      </c>
-      <c r="C24" t="s">
-        <v>167</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="E24">
-        <v>6</v>
-      </c>
-      <c r="F24" t="s">
-        <v>395</v>
-      </c>
-      <c r="I24" t="s">
-        <v>402</v>
+      <c r="G24" s="2"/>
+      <c r="H24" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -9132,112 +9278,113 @@
     <hyperlink ref="D20" r:id="rId19"/>
     <hyperlink ref="D21" r:id="rId20"/>
     <hyperlink ref="D22" r:id="rId21"/>
-    <hyperlink ref="D23" r:id="rId22"/>
-    <hyperlink ref="D24" r:id="rId23"/>
-    <hyperlink ref="D25" r:id="rId24"/>
-    <hyperlink ref="D26" r:id="rId25"/>
-    <hyperlink ref="D27" r:id="rId26"/>
-    <hyperlink ref="D28" r:id="rId27"/>
-    <hyperlink ref="D29" r:id="rId28"/>
-    <hyperlink ref="D30" r:id="rId29"/>
-    <hyperlink ref="D31" r:id="rId30"/>
-    <hyperlink ref="D32" r:id="rId31"/>
-    <hyperlink ref="D33" r:id="rId32"/>
-    <hyperlink ref="D34" r:id="rId33"/>
-    <hyperlink ref="D35" r:id="rId34"/>
-    <hyperlink ref="D36" r:id="rId35"/>
-    <hyperlink ref="D37" r:id="rId36"/>
-    <hyperlink ref="D38" r:id="rId37"/>
-    <hyperlink ref="D39" r:id="rId38"/>
-    <hyperlink ref="D40" r:id="rId39"/>
-    <hyperlink ref="D41" r:id="rId40"/>
-    <hyperlink ref="D42" r:id="rId41"/>
-    <hyperlink ref="D43" r:id="rId42"/>
-    <hyperlink ref="D44" r:id="rId43"/>
-    <hyperlink ref="D45" r:id="rId44"/>
-    <hyperlink ref="D46" r:id="rId45"/>
-    <hyperlink ref="D47" r:id="rId46"/>
-    <hyperlink ref="D48" r:id="rId47"/>
-    <hyperlink ref="D49" r:id="rId48"/>
-    <hyperlink ref="D50" r:id="rId49"/>
-    <hyperlink ref="D51" r:id="rId50"/>
-    <hyperlink ref="D52" r:id="rId51"/>
-    <hyperlink ref="D53" r:id="rId52"/>
-    <hyperlink ref="D54" r:id="rId53"/>
-    <hyperlink ref="D55" r:id="rId54"/>
-    <hyperlink ref="D56" r:id="rId55"/>
-    <hyperlink ref="D57" r:id="rId56"/>
-    <hyperlink ref="D58" r:id="rId57"/>
-    <hyperlink ref="D59" r:id="rId58"/>
-    <hyperlink ref="D60" r:id="rId59"/>
-    <hyperlink ref="D61" r:id="rId60"/>
-    <hyperlink ref="D62" r:id="rId61"/>
-    <hyperlink ref="D63" r:id="rId62"/>
-    <hyperlink ref="D64" r:id="rId63"/>
-    <hyperlink ref="D65" r:id="rId64"/>
-    <hyperlink ref="D66" r:id="rId65"/>
-    <hyperlink ref="D67" r:id="rId66"/>
-    <hyperlink ref="D68" r:id="rId67"/>
-    <hyperlink ref="D69" r:id="rId68"/>
-    <hyperlink ref="D70" r:id="rId69"/>
-    <hyperlink ref="D71" r:id="rId70"/>
-    <hyperlink ref="D72" r:id="rId71"/>
-    <hyperlink ref="D73" r:id="rId72"/>
-    <hyperlink ref="D74" r:id="rId73"/>
-    <hyperlink ref="D75" r:id="rId74"/>
-    <hyperlink ref="D76" r:id="rId75"/>
-    <hyperlink ref="D77" r:id="rId76"/>
-    <hyperlink ref="D78" r:id="rId77"/>
-    <hyperlink ref="D79" r:id="rId78"/>
-    <hyperlink ref="D80" r:id="rId79"/>
-    <hyperlink ref="D81" r:id="rId80"/>
-    <hyperlink ref="D82" r:id="rId81"/>
-    <hyperlink ref="D83" r:id="rId82"/>
-    <hyperlink ref="D84" r:id="rId83"/>
-    <hyperlink ref="D85" r:id="rId84"/>
-    <hyperlink ref="D86" r:id="rId85"/>
-    <hyperlink ref="D87" r:id="rId86"/>
-    <hyperlink ref="D88" r:id="rId87"/>
-    <hyperlink ref="D89" r:id="rId88"/>
-    <hyperlink ref="D90" r:id="rId89"/>
-    <hyperlink ref="D91" r:id="rId90"/>
-    <hyperlink ref="D92" r:id="rId91"/>
-    <hyperlink ref="D93" r:id="rId92"/>
-    <hyperlink ref="D94" r:id="rId93"/>
-    <hyperlink ref="D95" r:id="rId94"/>
-    <hyperlink ref="D96" r:id="rId95"/>
-    <hyperlink ref="D97" r:id="rId96"/>
-    <hyperlink ref="D98" r:id="rId97"/>
-    <hyperlink ref="D99" r:id="rId98"/>
-    <hyperlink ref="D100" r:id="rId99"/>
-    <hyperlink ref="D101" r:id="rId100"/>
-    <hyperlink ref="D102" r:id="rId101"/>
-    <hyperlink ref="D103" r:id="rId102"/>
-    <hyperlink ref="D104" r:id="rId103"/>
-    <hyperlink ref="D105" r:id="rId104"/>
-    <hyperlink ref="D106" r:id="rId105"/>
-    <hyperlink ref="D107" r:id="rId106"/>
-    <hyperlink ref="D108" r:id="rId107"/>
-    <hyperlink ref="D109" r:id="rId108"/>
-    <hyperlink ref="D110" r:id="rId109"/>
-    <hyperlink ref="D111" r:id="rId110"/>
-    <hyperlink ref="D112" r:id="rId111"/>
-    <hyperlink ref="D113" r:id="rId112"/>
-    <hyperlink ref="D114" r:id="rId113"/>
-    <hyperlink ref="D115" r:id="rId114"/>
-    <hyperlink ref="D116" r:id="rId115"/>
-    <hyperlink ref="D117" r:id="rId116"/>
-    <hyperlink ref="D118" r:id="rId117"/>
-    <hyperlink ref="D119" r:id="rId118"/>
-    <hyperlink ref="D120" r:id="rId119"/>
-    <hyperlink ref="D121" r:id="rId120"/>
-    <hyperlink ref="D122" r:id="rId121"/>
-    <hyperlink ref="D123" r:id="rId122"/>
-    <hyperlink ref="D124" r:id="rId123"/>
-    <hyperlink ref="D125" r:id="rId124"/>
-    <hyperlink ref="D126" r:id="rId125"/>
+    <hyperlink ref="D24" r:id="rId22"/>
+    <hyperlink ref="D25" r:id="rId23"/>
+    <hyperlink ref="D26" r:id="rId24"/>
+    <hyperlink ref="D27" r:id="rId25"/>
+    <hyperlink ref="D28" r:id="rId26"/>
+    <hyperlink ref="D29" r:id="rId27"/>
+    <hyperlink ref="D30" r:id="rId28"/>
+    <hyperlink ref="D31" r:id="rId29"/>
+    <hyperlink ref="D32" r:id="rId30"/>
+    <hyperlink ref="D33" r:id="rId31"/>
+    <hyperlink ref="D34" r:id="rId32"/>
+    <hyperlink ref="D35" r:id="rId33"/>
+    <hyperlink ref="D36" r:id="rId34"/>
+    <hyperlink ref="D37" r:id="rId35"/>
+    <hyperlink ref="D38" r:id="rId36"/>
+    <hyperlink ref="D39" r:id="rId37"/>
+    <hyperlink ref="D40" r:id="rId38"/>
+    <hyperlink ref="D41" r:id="rId39"/>
+    <hyperlink ref="D42" r:id="rId40"/>
+    <hyperlink ref="D43" r:id="rId41"/>
+    <hyperlink ref="D44" r:id="rId42"/>
+    <hyperlink ref="D45" r:id="rId43"/>
+    <hyperlink ref="D46" r:id="rId44"/>
+    <hyperlink ref="D47" r:id="rId45"/>
+    <hyperlink ref="D48" r:id="rId46"/>
+    <hyperlink ref="D49" r:id="rId47"/>
+    <hyperlink ref="D50" r:id="rId48"/>
+    <hyperlink ref="D51" r:id="rId49"/>
+    <hyperlink ref="D52" r:id="rId50"/>
+    <hyperlink ref="D53" r:id="rId51"/>
+    <hyperlink ref="D54" r:id="rId52"/>
+    <hyperlink ref="D55" r:id="rId53"/>
+    <hyperlink ref="D56" r:id="rId54"/>
+    <hyperlink ref="D57" r:id="rId55"/>
+    <hyperlink ref="D58" r:id="rId56"/>
+    <hyperlink ref="D59" r:id="rId57"/>
+    <hyperlink ref="D60" r:id="rId58"/>
+    <hyperlink ref="D61" r:id="rId59"/>
+    <hyperlink ref="D62" r:id="rId60"/>
+    <hyperlink ref="D63" r:id="rId61"/>
+    <hyperlink ref="D64" r:id="rId62"/>
+    <hyperlink ref="D65" r:id="rId63"/>
+    <hyperlink ref="D66" r:id="rId64"/>
+    <hyperlink ref="D67" r:id="rId65"/>
+    <hyperlink ref="D68" r:id="rId66"/>
+    <hyperlink ref="D69" r:id="rId67"/>
+    <hyperlink ref="D70" r:id="rId68"/>
+    <hyperlink ref="D71" r:id="rId69"/>
+    <hyperlink ref="D72" r:id="rId70"/>
+    <hyperlink ref="D73" r:id="rId71"/>
+    <hyperlink ref="D74" r:id="rId72"/>
+    <hyperlink ref="D75" r:id="rId73"/>
+    <hyperlink ref="D76" r:id="rId74"/>
+    <hyperlink ref="D77" r:id="rId75"/>
+    <hyperlink ref="D78" r:id="rId76"/>
+    <hyperlink ref="D79" r:id="rId77"/>
+    <hyperlink ref="D80" r:id="rId78"/>
+    <hyperlink ref="D81" r:id="rId79"/>
+    <hyperlink ref="D82" r:id="rId80"/>
+    <hyperlink ref="D83" r:id="rId81"/>
+    <hyperlink ref="D84" r:id="rId82"/>
+    <hyperlink ref="D85" r:id="rId83"/>
+    <hyperlink ref="D86" r:id="rId84"/>
+    <hyperlink ref="D87" r:id="rId85"/>
+    <hyperlink ref="D88" r:id="rId86"/>
+    <hyperlink ref="D89" r:id="rId87"/>
+    <hyperlink ref="D90" r:id="rId88"/>
+    <hyperlink ref="D91" r:id="rId89"/>
+    <hyperlink ref="D92" r:id="rId90"/>
+    <hyperlink ref="D93" r:id="rId91"/>
+    <hyperlink ref="D94" r:id="rId92"/>
+    <hyperlink ref="D95" r:id="rId93"/>
+    <hyperlink ref="D96" r:id="rId94"/>
+    <hyperlink ref="D97" r:id="rId95"/>
+    <hyperlink ref="D98" r:id="rId96"/>
+    <hyperlink ref="D99" r:id="rId97"/>
+    <hyperlink ref="D100" r:id="rId98"/>
+    <hyperlink ref="D101" r:id="rId99"/>
+    <hyperlink ref="D102" r:id="rId100"/>
+    <hyperlink ref="D103" r:id="rId101"/>
+    <hyperlink ref="D104" r:id="rId102"/>
+    <hyperlink ref="D105" r:id="rId103"/>
+    <hyperlink ref="D106" r:id="rId104"/>
+    <hyperlink ref="D107" r:id="rId105"/>
+    <hyperlink ref="D108" r:id="rId106"/>
+    <hyperlink ref="D109" r:id="rId107"/>
+    <hyperlink ref="D110" r:id="rId108"/>
+    <hyperlink ref="D111" r:id="rId109"/>
+    <hyperlink ref="D112" r:id="rId110"/>
+    <hyperlink ref="D113" r:id="rId111"/>
+    <hyperlink ref="D114" r:id="rId112"/>
+    <hyperlink ref="D115" r:id="rId113"/>
+    <hyperlink ref="D116" r:id="rId114"/>
+    <hyperlink ref="D117" r:id="rId115"/>
+    <hyperlink ref="D118" r:id="rId116"/>
+    <hyperlink ref="D119" r:id="rId117"/>
+    <hyperlink ref="D120" r:id="rId118"/>
+    <hyperlink ref="D121" r:id="rId119"/>
+    <hyperlink ref="D122" r:id="rId120"/>
+    <hyperlink ref="D123" r:id="rId121"/>
+    <hyperlink ref="D124" r:id="rId122"/>
+    <hyperlink ref="D125" r:id="rId123"/>
+    <hyperlink ref="D126" r:id="rId124"/>
+    <hyperlink ref="D23" r:id="rId125"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId126"/>
 </worksheet>
 </file>
 
@@ -9245,6 +9392,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K1155"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" customWidth="1"/>
+    <col min="8" max="8" width="255.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="135" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
125 leis revisadas manualmente para formação do dataset ouro - parte Filipe
</commit_message>
<xml_diff>
--- a/avaliacao/Filipe/ouro_Filipe.xlsx
+++ b/avaliacao/Filipe/ouro_Filipe.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8768" uniqueCount="1929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8879" uniqueCount="1930">
   <si>
     <t>campo</t>
   </si>
@@ -5803,6 +5803,9 @@
   </si>
   <si>
     <t>O artigo 10, inciso I estava com o inciso II unido no texto, sendo que era apenas uma referência no texto para indicar o inciso II.</t>
+  </si>
+  <si>
+    <t>No Artigo 3º, o texto do Inciso III estava unido no texto do Inciso II e não era contalizado como fragmento.</t>
   </si>
 </sst>
 </file>
@@ -5861,9 +5864,8 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
@@ -6232,6 +6234,7 @@
     <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.42578125" customWidth="1"/>
     <col min="4" max="4" width="112.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" customWidth="1"/>
     <col min="7" max="7" width="217" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -6268,2991 +6271,3416 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>1936</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>8</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2" t="s">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>1937</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <v>6</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>1926</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>1923</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="2" t="s">
         <v>1925</v>
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>1935</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <v>4</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>1927</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>1923</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="2" t="s">
         <v>1925</v>
       </c>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>1937</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>2</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>1927</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>1923</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>1925</v>
       </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>1937</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <v>2</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>1927</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="2" t="s">
         <v>1923</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>1925</v>
       </c>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>1951</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>25</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <v>1955</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>9</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>1957</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>21</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>1964</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>52</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2" t="s">
+      <c r="G10" s="1"/>
+      <c r="H10" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>1966</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>45</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>1968</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>10</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2" t="s">
+      <c r="G12" s="1"/>
+      <c r="H12" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <v>1971</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>7</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2" t="s">
+      <c r="G13" s="1"/>
+      <c r="H13" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <v>1973</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>44</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2" t="s">
+      <c r="G14" s="1"/>
+      <c r="H14" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <v>1948</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>6</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2" t="s">
+      <c r="G15" s="1"/>
+      <c r="H15" s="1" t="s">
         <v>1923</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="1" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <v>1975</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>13</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="6" t="s">
+      <c r="G16" s="1"/>
+      <c r="H16" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I16" s="6" t="s">
+      <c r="I16" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="1">
         <v>1977</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>8</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G17" s="2"/>
-      <c r="H17" s="6" t="s">
+      <c r="G17" s="1"/>
+      <c r="H17" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <v>1979</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>7</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G18" s="2"/>
-      <c r="H18" s="6" t="s">
+      <c r="G18" s="1"/>
+      <c r="H18" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I18" s="6" t="s">
+      <c r="I18" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <v>1981</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>7</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G19" s="2"/>
-      <c r="H19" s="6" t="s">
+      <c r="G19" s="1"/>
+      <c r="H19" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>1981</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="4" t="s">
         <v>288</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>13</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="G20" s="2"/>
-      <c r="H20" s="6" t="s">
+      <c r="G20" s="1"/>
+      <c r="H20" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="21" spans="1:9">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>1984</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>6</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="6" t="s">
+      <c r="G21" s="1"/>
+      <c r="H21" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="I21" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>1985</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>8</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="G22" s="2"/>
-      <c r="H22" s="6" t="s">
+      <c r="G22" s="1"/>
+      <c r="H22" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="23" spans="1:9">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23" s="2">
         <v>1986</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="2">
         <v>57</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" s="2" t="s">
         <v>1928</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="2" t="s">
         <v>1923</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I23" s="2" t="s">
         <v>1925</v>
       </c>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>1987</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>6</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="6" t="s">
+      <c r="G24" s="1"/>
+      <c r="H24" s="5" t="s">
         <v>1923</v>
       </c>
-      <c r="I24" s="6" t="s">
+      <c r="I24" s="5" t="s">
         <v>1924</v>
       </c>
     </row>
     <row r="25" spans="1:9">
-      <c r="A25" t="s">
+      <c r="A25" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>1949</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="1">
         <v>23</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I25" t="s">
-        <v>402</v>
+      <c r="G25" s="1"/>
+      <c r="H25" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="26" spans="1:9">
-      <c r="A26" t="s">
+      <c r="A26" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="1">
         <v>1950</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="4" t="s">
         <v>294</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="1">
         <v>4</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I26" t="s">
-        <v>402</v>
+      <c r="G26" s="1"/>
+      <c r="H26" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" t="s">
+      <c r="A27" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="1">
         <v>1955</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="1">
         <v>3</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I27" t="s">
-        <v>402</v>
+      <c r="G27" s="1"/>
+      <c r="H27" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="28" spans="1:9">
-      <c r="A28" t="s">
+      <c r="A28" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="1">
         <v>1956</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="1">
         <v>5</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I28" t="s">
-        <v>402</v>
+      <c r="G28" s="1"/>
+      <c r="H28" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="29" spans="1:9">
-      <c r="A29" t="s">
+      <c r="A29" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="1">
         <v>1960</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="1">
         <v>3</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I29" t="s">
-        <v>402</v>
+      <c r="G29" s="1"/>
+      <c r="H29" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="30" spans="1:9">
-      <c r="A30" t="s">
+      <c r="A30" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="1">
         <v>1960</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="1">
         <v>4</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="I30" t="s">
-        <v>402</v>
+      <c r="G30" s="1"/>
+      <c r="H30" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="31" spans="1:9">
-      <c r="A31" t="s">
+      <c r="A31" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="1">
         <v>1966</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="1">
         <v>4</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I31" t="s">
-        <v>402</v>
+      <c r="G31" s="1"/>
+      <c r="H31" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="32" spans="1:9">
-      <c r="A32" t="s">
+      <c r="A32" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="1">
         <v>1966</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D32" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="1">
         <v>3</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I32" t="s">
-        <v>402</v>
+      <c r="G32" s="1"/>
+      <c r="H32" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="33" spans="1:9">
-      <c r="A33" t="s">
+      <c r="A33" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="1">
         <v>1967</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="1">
         <v>3</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I33" t="s">
-        <v>402</v>
+      <c r="G33" s="1"/>
+      <c r="H33" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="34" spans="1:9">
-      <c r="A34" t="s">
+      <c r="A34" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="1">
         <v>1967</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D34" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="1">
         <v>5</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I34" t="s">
-        <v>402</v>
+      <c r="G34" s="1"/>
+      <c r="H34" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="35" spans="1:9">
-      <c r="A35" t="s">
+      <c r="A35" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="1">
         <v>1968</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D35" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="1">
         <v>4</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I35" t="s">
-        <v>402</v>
+      <c r="G35" s="1"/>
+      <c r="H35" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="36" spans="1:9">
-      <c r="A36" t="s">
+      <c r="A36" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="1">
         <v>1968</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="1">
         <v>5</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I36" t="s">
-        <v>402</v>
+      <c r="G36" s="1"/>
+      <c r="H36" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="37" spans="1:9">
-      <c r="A37" t="s">
+      <c r="A37" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="1">
         <v>1968</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" s="4" t="s">
         <v>305</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="1">
         <v>3</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I37" t="s">
-        <v>402</v>
+      <c r="G37" s="1"/>
+      <c r="H37" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="38" spans="1:9">
-      <c r="A38" t="s">
+      <c r="A38" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="1">
         <v>1968</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="1">
         <v>5</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="I38" t="s">
-        <v>402</v>
+      <c r="H38" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="39" spans="1:9">
-      <c r="A39" t="s">
+      <c r="A39" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="1">
         <v>1974</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="1">
         <v>3</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I39" t="s">
-        <v>402</v>
+      <c r="G39" s="1"/>
+      <c r="H39" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="40" spans="1:9">
-      <c r="A40" t="s">
+      <c r="A40" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="1">
         <v>1974</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D40" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="1">
         <v>3</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I40" t="s">
-        <v>402</v>
+      <c r="G40" s="1"/>
+      <c r="H40" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="41" spans="1:9">
-      <c r="A41" t="s">
+      <c r="A41" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="1">
         <v>1975</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D41" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="1">
         <v>3</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I41" t="s">
-        <v>402</v>
+      <c r="G41" s="1"/>
+      <c r="H41" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="42" spans="1:9">
-      <c r="A42" t="s">
+      <c r="A42" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="1">
         <v>1981</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D42" s="4" t="s">
         <v>310</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="1">
         <v>5</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="I42" t="s">
-        <v>402</v>
+      <c r="G42" s="1"/>
+      <c r="H42" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="43" spans="1:9">
-      <c r="A43" t="s">
+      <c r="A43" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="1">
         <v>1981</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D43" s="4" t="s">
         <v>311</v>
       </c>
-      <c r="E43">
+      <c r="E43" s="1">
         <v>3</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="I43" t="s">
-        <v>402</v>
+      <c r="G43" s="1"/>
+      <c r="H43" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="44" spans="1:9">
-      <c r="A44" t="s">
+      <c r="A44" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="1">
         <v>1982</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D44" s="4" t="s">
         <v>312</v>
       </c>
-      <c r="E44">
+      <c r="E44" s="1">
         <v>4</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I44" t="s">
-        <v>402</v>
+      <c r="G44" s="1"/>
+      <c r="H44" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="45" spans="1:9">
-      <c r="A45" t="s">
+      <c r="A45" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="1">
         <v>1983</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D45" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="1">
         <v>4</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I45" t="s">
-        <v>402</v>
+      <c r="G45" s="1"/>
+      <c r="H45" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="46" spans="1:9">
-      <c r="A46" t="s">
+      <c r="A46" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="1">
         <v>1983</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D46" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="E46">
+      <c r="E46" s="1">
         <v>5</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I46" t="s">
-        <v>402</v>
+      <c r="G46" s="1"/>
+      <c r="H46" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="47" spans="1:9">
-      <c r="A47" t="s">
+      <c r="A47" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="1">
         <v>1984</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D47" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="E47">
+      <c r="E47" s="1">
         <v>5</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I47" t="s">
-        <v>402</v>
+      <c r="G47" s="1"/>
+      <c r="H47" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="48" spans="1:9">
-      <c r="A48" t="s">
+      <c r="A48" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="1">
         <v>1985</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D48" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="E48">
+      <c r="E48" s="1">
         <v>4</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I48" t="s">
-        <v>402</v>
+      <c r="G48" s="1"/>
+      <c r="H48" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="49" spans="1:9">
-      <c r="A49" t="s">
+      <c r="A49" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="1">
         <v>1949</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D49" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="E49">
+      <c r="E49" s="1">
         <v>4</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I49" t="s">
-        <v>402</v>
+      <c r="G49" s="1"/>
+      <c r="H49" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="50" spans="1:9">
-      <c r="A50" t="s">
+      <c r="A50" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="1">
         <v>1949</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="D50" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="E50">
+      <c r="E50" s="1">
         <v>3</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F50" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I50" t="s">
-        <v>402</v>
+      <c r="G50" s="1"/>
+      <c r="H50" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="51" spans="1:9">
-      <c r="A51" t="s">
+      <c r="A51" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="1">
         <v>1950</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="D51" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="E51">
+      <c r="E51" s="1">
         <v>2</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F51" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I51" t="s">
-        <v>402</v>
+      <c r="G51" s="1"/>
+      <c r="H51" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="52" spans="1:9">
-      <c r="A52" t="s">
+      <c r="A52" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="1">
         <v>1951</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="D52" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="E52">
+      <c r="E52" s="1">
         <v>3</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F52" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I52" t="s">
-        <v>402</v>
+      <c r="G52" s="1"/>
+      <c r="H52" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="53" spans="1:9">
-      <c r="A53" t="s">
+      <c r="A53" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="1">
         <v>1952</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="D53" s="1" t="s">
+      <c r="D53" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="E53">
+      <c r="E53" s="1">
         <v>3</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I53" t="s">
-        <v>402</v>
+      <c r="G53" s="1"/>
+      <c r="H53" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="54" spans="1:9">
-      <c r="A54" t="s">
+      <c r="A54" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="1">
         <v>1952</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="D54" s="1" t="s">
+      <c r="D54" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="E54">
+      <c r="E54" s="1">
         <v>3</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F54" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I54" t="s">
-        <v>402</v>
+      <c r="G54" s="1"/>
+      <c r="H54" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="55" spans="1:9">
-      <c r="A55" t="s">
+      <c r="A55" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="1">
         <v>1952</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="D55" s="1" t="s">
+      <c r="D55" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="E55">
+      <c r="E55" s="1">
         <v>2</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F55" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I55" t="s">
-        <v>402</v>
+      <c r="G55" s="1"/>
+      <c r="H55" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="56" spans="1:9">
-      <c r="A56" t="s">
+      <c r="A56" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="1">
         <v>1947</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D56" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="E56">
+      <c r="E56" s="1">
         <v>2</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F56" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I56" t="s">
-        <v>402</v>
+      <c r="G56" s="1"/>
+      <c r="H56" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="57" spans="1:9">
-      <c r="A57" t="s">
+      <c r="A57" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="1">
         <v>1953</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D57" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="E57">
+      <c r="E57" s="1">
         <v>3</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F57" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I57" t="s">
-        <v>402</v>
+      <c r="G57" s="1"/>
+      <c r="H57" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I57" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="58" spans="1:9">
-      <c r="A58" t="s">
+      <c r="A58" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="1">
         <v>1955</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="D58" s="1" t="s">
+      <c r="D58" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="E58">
+      <c r="E58" s="1">
         <v>2</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F58" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I58" t="s">
-        <v>402</v>
+      <c r="G58" s="1"/>
+      <c r="H58" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I58" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="59" spans="1:9">
-      <c r="A59" t="s">
+      <c r="A59" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B59">
+      <c r="B59" s="1">
         <v>1957</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D59" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="E59">
+      <c r="E59" s="1">
         <v>2</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F59" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I59" t="s">
-        <v>402</v>
+      <c r="G59" s="1"/>
+      <c r="H59" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I59" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="60" spans="1:9">
-      <c r="A60" t="s">
+      <c r="A60" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="1">
         <v>1959</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D60" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="1">
         <v>2</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F60" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I60" t="s">
-        <v>402</v>
+      <c r="G60" s="1"/>
+      <c r="H60" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="61" spans="1:9">
-      <c r="A61" t="s">
+      <c r="A61" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B61">
+      <c r="B61" s="1">
         <v>1948</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C61" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="D61" s="1" t="s">
+      <c r="D61" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="E61">
+      <c r="E61" s="1">
         <v>2</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I61" t="s">
-        <v>402</v>
+      <c r="G61" s="1"/>
+      <c r="H61" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I61" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="62" spans="1:9">
-      <c r="A62" t="s">
+      <c r="A62" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B62">
+      <c r="B62" s="1">
         <v>1962</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C62" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="D62" s="1" t="s">
+      <c r="D62" s="4" t="s">
         <v>330</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="1">
         <v>2</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F62" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I62" t="s">
-        <v>402</v>
+      <c r="G62" s="1"/>
+      <c r="H62" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I62" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="63" spans="1:9">
-      <c r="A63" t="s">
+      <c r="A63" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="1">
         <v>1963</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C63" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="D63" s="1" t="s">
+      <c r="D63" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="E63">
+      <c r="E63" s="1">
         <v>2</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F63" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I63" t="s">
-        <v>402</v>
+      <c r="G63" s="1"/>
+      <c r="H63" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I63" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="64" spans="1:9">
-      <c r="A64" t="s">
+      <c r="A64" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="1">
         <v>1965</v>
       </c>
-      <c r="C64" t="s">
+      <c r="C64" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="D64" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="E64">
+      <c r="E64" s="1">
         <v>2</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I64" t="s">
-        <v>402</v>
+      <c r="G64" s="1"/>
+      <c r="H64" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I64" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="65" spans="1:9">
-      <c r="A65" t="s">
+      <c r="A65" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="1">
         <v>1974</v>
       </c>
-      <c r="C65" t="s">
+      <c r="C65" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="D65" s="1" t="s">
+      <c r="D65" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="E65">
+      <c r="E65" s="1">
         <v>2</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F65" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I65" t="s">
-        <v>402</v>
+      <c r="G65" s="1"/>
+      <c r="H65" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I65" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="66" spans="1:9">
-      <c r="A66" t="s">
+      <c r="A66" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B66">
+      <c r="B66" s="1">
         <v>1983</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C66" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="D66" s="1" t="s">
+      <c r="D66" s="4" t="s">
         <v>334</v>
       </c>
-      <c r="E66">
+      <c r="E66" s="1">
         <v>2</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F66" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I66" t="s">
-        <v>402</v>
+      <c r="G66" s="1"/>
+      <c r="H66" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I66" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="67" spans="1:9">
-      <c r="A67" t="s">
+      <c r="A67" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="1">
         <v>1947</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C67" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="D67" s="1" t="s">
+      <c r="D67" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="E67">
+      <c r="E67" s="1">
         <v>2</v>
       </c>
-      <c r="F67" t="s">
+      <c r="F67" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I67" t="s">
-        <v>402</v>
+      <c r="G67" s="1"/>
+      <c r="H67" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I67" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="68" spans="1:9">
-      <c r="A68" t="s">
+      <c r="A68" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="1">
         <v>2002</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C68" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="D68" s="4" t="s">
         <v>336</v>
       </c>
-      <c r="E68">
+      <c r="E68" s="1">
         <v>6</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F68" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I68" t="s">
-        <v>402</v>
+      <c r="G68" s="1"/>
+      <c r="H68" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I68" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="69" spans="1:9">
-      <c r="A69" t="s">
+      <c r="A69" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B69">
+      <c r="B69" s="1">
         <v>2004</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C69" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="D69" s="1" t="s">
+      <c r="D69" s="4" t="s">
         <v>337</v>
       </c>
-      <c r="E69">
+      <c r="E69" s="1">
         <v>6</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F69" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I69" t="s">
-        <v>402</v>
+      <c r="G69" s="1"/>
+      <c r="H69" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I69" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="70" spans="1:9">
-      <c r="A70" t="s">
+      <c r="A70" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B70">
+      <c r="B70" s="2">
         <v>2004</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C70" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D70" s="1" t="s">
+      <c r="D70" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="E70">
-        <v>21</v>
-      </c>
-      <c r="F70" t="s">
+      <c r="E70" s="2">
+        <v>22</v>
+      </c>
+      <c r="F70" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I70" t="s">
-        <v>402</v>
+      <c r="G70" s="2" t="s">
+        <v>1929</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="71" spans="1:9">
-      <c r="A71" t="s">
+      <c r="A71" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B71">
+      <c r="B71" s="1">
         <v>2007</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C71" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="D71" s="1" t="s">
+      <c r="D71" s="4" t="s">
         <v>339</v>
       </c>
-      <c r="E71">
+      <c r="E71" s="1">
         <v>32</v>
       </c>
-      <c r="F71" t="s">
+      <c r="F71" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I71" t="s">
-        <v>402</v>
+      <c r="G71" s="1"/>
+      <c r="H71" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I71" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="72" spans="1:9">
-      <c r="A72" t="s">
+      <c r="A72" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B72">
+      <c r="B72" s="1">
         <v>2008</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C72" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="D72" s="1" t="s">
+      <c r="D72" s="4" t="s">
         <v>340</v>
       </c>
-      <c r="E72">
+      <c r="E72" s="1">
         <v>8</v>
       </c>
-      <c r="F72" t="s">
+      <c r="F72" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I72" t="s">
-        <v>402</v>
+      <c r="G72" s="1"/>
+      <c r="H72" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I72" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="73" spans="1:9">
-      <c r="A73" t="s">
+      <c r="A73" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B73">
+      <c r="B73" s="2">
         <v>2010</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C73" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="D73" s="1" t="s">
+      <c r="D73" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="E73">
+      <c r="E73" s="2">
         <v>6</v>
       </c>
-      <c r="F73" t="s">
+      <c r="F73" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I73" t="s">
-        <v>402</v>
+      <c r="G73" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="74" spans="1:9">
-      <c r="A74" t="s">
+      <c r="A74" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B74">
+      <c r="B74" s="2">
         <v>2010</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C74" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D74" s="1" t="s">
+      <c r="D74" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="E74">
+      <c r="E74" s="2">
         <v>27</v>
       </c>
-      <c r="F74" t="s">
+      <c r="F74" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I74" t="s">
-        <v>402</v>
+      <c r="G74" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="75" spans="1:9">
-      <c r="A75" t="s">
+      <c r="A75" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B75">
+      <c r="B75" s="1">
         <v>2016</v>
       </c>
-      <c r="C75" t="s">
+      <c r="C75" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="D75" s="1" t="s">
+      <c r="D75" s="4" t="s">
         <v>343</v>
       </c>
-      <c r="E75">
+      <c r="E75" s="1">
         <v>9</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F75" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I75" t="s">
-        <v>402</v>
+      <c r="G75" s="1"/>
+      <c r="H75" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I75" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="76" spans="1:9">
-      <c r="A76" t="s">
+      <c r="A76" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B76">
+      <c r="B76" s="1">
         <v>2017</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C76" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D76" s="1" t="s">
+      <c r="D76" s="4" t="s">
         <v>344</v>
       </c>
-      <c r="E76">
+      <c r="E76" s="1">
         <v>11</v>
       </c>
-      <c r="F76" t="s">
+      <c r="F76" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I76" t="s">
-        <v>402</v>
+      <c r="G76" s="1"/>
+      <c r="H76" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I76" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="77" spans="1:9">
-      <c r="A77" t="s">
+      <c r="A77" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B77">
+      <c r="B77" s="1">
         <v>2022</v>
       </c>
-      <c r="C77" t="s">
+      <c r="C77" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="D77" s="1" t="s">
+      <c r="D77" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="E77">
+      <c r="E77" s="1">
         <v>14</v>
       </c>
-      <c r="F77" t="s">
+      <c r="F77" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I77" t="s">
-        <v>402</v>
+      <c r="G77" s="1"/>
+      <c r="H77" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I77" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="78" spans="1:9">
-      <c r="A78" t="s">
+      <c r="A78" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B78">
+      <c r="B78" s="1">
         <v>2022</v>
       </c>
-      <c r="C78" t="s">
+      <c r="C78" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="D78" s="1" t="s">
+      <c r="D78" s="4" t="s">
         <v>346</v>
       </c>
-      <c r="E78">
+      <c r="E78" s="1">
         <v>10</v>
       </c>
-      <c r="F78" t="s">
+      <c r="F78" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I78" t="s">
-        <v>402</v>
+      <c r="G78" s="1"/>
+      <c r="H78" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I78" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="79" spans="1:9">
-      <c r="A79" t="s">
+      <c r="A79" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B79">
+      <c r="B79" s="1">
         <v>2025</v>
       </c>
-      <c r="C79" t="s">
+      <c r="C79" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D79" s="1" t="s">
+      <c r="D79" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="E79">
+      <c r="E79" s="1">
         <v>24</v>
       </c>
-      <c r="F79" t="s">
+      <c r="F79" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I79" t="s">
-        <v>402</v>
+      <c r="G79" s="1"/>
+      <c r="H79" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I79" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="80" spans="1:9">
-      <c r="A80" t="s">
+      <c r="A80" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B80">
+      <c r="B80" s="1">
         <v>2025</v>
       </c>
-      <c r="C80" t="s">
+      <c r="C80" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="D80" s="4" t="s">
         <v>348</v>
       </c>
-      <c r="E80">
+      <c r="E80" s="1">
         <v>6</v>
       </c>
-      <c r="F80" t="s">
+      <c r="F80" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I80" t="s">
-        <v>402</v>
+      <c r="G80" s="1"/>
+      <c r="H80" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I80" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="81" spans="1:9">
-      <c r="A81" t="s">
+      <c r="A81" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B81">
+      <c r="B81" s="1">
         <v>2026</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C81" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="D81" s="1" t="s">
+      <c r="D81" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="E81">
+      <c r="E81" s="1">
         <v>51</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F81" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="I81" t="s">
-        <v>402</v>
+      <c r="G81" s="1"/>
+      <c r="H81" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I81" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="82" spans="1:9">
-      <c r="A82" t="s">
+      <c r="A82" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B82">
+      <c r="B82" s="2">
         <v>1989</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C82" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="D82" s="1" t="s">
+      <c r="D82" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="E82">
+      <c r="E82" s="2">
         <v>31</v>
       </c>
-      <c r="F82" t="s">
+      <c r="F82" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I82" t="s">
-        <v>402</v>
+      <c r="G82" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I82" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="83" spans="1:9">
-      <c r="A83" t="s">
+      <c r="A83" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B83">
+      <c r="B83" s="1">
         <v>1989</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C83" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D83" s="4" t="s">
         <v>351</v>
       </c>
-      <c r="E83">
+      <c r="E83" s="1">
         <v>5</v>
       </c>
-      <c r="F83" t="s">
+      <c r="F83" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I83" t="s">
-        <v>402</v>
+      <c r="G83" s="1"/>
+      <c r="H83" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I83" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="84" spans="1:9">
-      <c r="A84" t="s">
+      <c r="A84" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B84">
+      <c r="B84" s="1">
         <v>1990</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C84" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D84" s="4" t="s">
         <v>352</v>
       </c>
-      <c r="E84">
+      <c r="E84" s="1">
         <v>6</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F84" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I84" t="s">
-        <v>402</v>
+      <c r="G84" s="1"/>
+      <c r="H84" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I84" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="85" spans="1:9">
-      <c r="A85" t="s">
+      <c r="A85" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B85">
+      <c r="B85" s="1">
         <v>1992</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C85" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="D85" s="1" t="s">
+      <c r="D85" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E85">
+      <c r="E85" s="1">
         <v>5</v>
       </c>
-      <c r="F85" t="s">
+      <c r="F85" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I85" t="s">
-        <v>402</v>
+      <c r="G85" s="1"/>
+      <c r="H85" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I85" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="86" spans="1:9">
-      <c r="A86" t="s">
+      <c r="A86" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B86">
+      <c r="B86" s="1">
         <v>1992</v>
       </c>
-      <c r="C86" t="s">
+      <c r="C86" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="D86" s="4" t="s">
         <v>354</v>
       </c>
-      <c r="E86">
+      <c r="E86" s="1">
         <v>10</v>
       </c>
-      <c r="F86" t="s">
+      <c r="F86" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I86" t="s">
-        <v>402</v>
+      <c r="G86" s="1"/>
+      <c r="H86" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I86" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="87" spans="1:9">
-      <c r="A87" t="s">
+      <c r="A87" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B87">
+      <c r="B87" s="1">
         <v>1993</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C87" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="D87" s="1" t="s">
+      <c r="D87" s="4" t="s">
         <v>355</v>
       </c>
-      <c r="E87">
+      <c r="E87" s="1">
         <v>60</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F87" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I87" t="s">
-        <v>402</v>
+      <c r="G87" s="1"/>
+      <c r="H87" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I87" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="88" spans="1:9">
-      <c r="A88" t="s">
+      <c r="A88" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B88">
+      <c r="B88" s="1">
         <v>1996</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C88" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="D88" s="1" t="s">
+      <c r="D88" s="4" t="s">
         <v>356</v>
       </c>
-      <c r="E88">
+      <c r="E88" s="1">
         <v>143</v>
       </c>
-      <c r="F88" t="s">
+      <c r="F88" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I88" t="s">
-        <v>402</v>
+      <c r="G88" s="1"/>
+      <c r="H88" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I88" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="89" spans="1:9">
-      <c r="A89" t="s">
+      <c r="A89" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B89">
+      <c r="B89" s="1">
         <v>1999</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C89" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="D89" s="1" t="s">
+      <c r="D89" s="4" t="s">
         <v>357</v>
       </c>
-      <c r="E89">
+      <c r="E89" s="1">
         <v>27</v>
       </c>
-      <c r="F89" t="s">
+      <c r="F89" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I89" t="s">
-        <v>402</v>
+      <c r="G89" s="1"/>
+      <c r="H89" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I89" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="90" spans="1:9">
-      <c r="A90" t="s">
+      <c r="A90" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B90">
+      <c r="B90" s="1">
         <v>2001</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C90" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="D90" s="1" t="s">
+      <c r="D90" s="4" t="s">
         <v>358</v>
       </c>
-      <c r="E90">
+      <c r="E90" s="1">
         <v>4</v>
       </c>
-      <c r="F90" t="s">
+      <c r="F90" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I90" t="s">
-        <v>402</v>
+      <c r="G90" s="1"/>
+      <c r="H90" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I90" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="91" spans="1:9">
-      <c r="A91" t="s">
+      <c r="A91" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B91">
+      <c r="B91" s="1">
         <v>2005</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C91" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="D91" s="1" t="s">
+      <c r="D91" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="E91">
+      <c r="E91" s="1">
         <v>5</v>
       </c>
-      <c r="F91" t="s">
+      <c r="F91" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I91" t="s">
-        <v>402</v>
+      <c r="G91" s="1"/>
+      <c r="H91" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I91" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="92" spans="1:9">
-      <c r="A92" t="s">
+      <c r="A92" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B92">
+      <c r="B92" s="1">
         <v>2007</v>
       </c>
-      <c r="C92" t="s">
+      <c r="C92" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="D92" s="1" t="s">
+      <c r="D92" s="4" t="s">
         <v>360</v>
       </c>
-      <c r="E92">
+      <c r="E92" s="1">
         <v>4</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F92" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I92" t="s">
-        <v>402</v>
+      <c r="G92" s="1"/>
+      <c r="H92" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I92" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="93" spans="1:9">
-      <c r="A93" t="s">
+      <c r="A93" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B93">
+      <c r="B93" s="1">
         <v>2008</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C93" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="D93" s="1" t="s">
+      <c r="D93" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="E93">
+      <c r="E93" s="1">
         <v>5</v>
       </c>
-      <c r="F93" t="s">
+      <c r="F93" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I93" t="s">
-        <v>402</v>
+      <c r="G93" s="1"/>
+      <c r="H93" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I93" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="94" spans="1:9">
-      <c r="A94" t="s">
+      <c r="A94" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B94">
+      <c r="B94" s="2">
         <v>2009</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C94" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="D94" s="1" t="s">
+      <c r="D94" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="E94">
+      <c r="E94" s="2">
         <v>4</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F94" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I94" t="s">
-        <v>402</v>
+      <c r="G94" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I94" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="95" spans="1:9">
-      <c r="A95" t="s">
+      <c r="A95" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B95">
+      <c r="B95" s="2">
         <v>2009</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C95" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="D95" s="1" t="s">
+      <c r="D95" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="E95">
+      <c r="E95" s="2">
         <v>4</v>
       </c>
-      <c r="F95" t="s">
+      <c r="F95" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I95" t="s">
-        <v>402</v>
+      <c r="G95" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H95" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I95" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="96" spans="1:9">
-      <c r="A96" t="s">
+      <c r="A96" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B96">
+      <c r="B96" s="2">
         <v>2011</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C96" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="D96" s="1" t="s">
+      <c r="D96" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="E96">
+      <c r="E96" s="2">
         <v>4</v>
       </c>
-      <c r="F96" t="s">
+      <c r="F96" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I96" t="s">
-        <v>402</v>
+      <c r="G96" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H96" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I96" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="97" spans="1:9">
-      <c r="A97" t="s">
+      <c r="A97" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B97">
+      <c r="B97" s="1">
         <v>2016</v>
       </c>
-      <c r="C97" t="s">
+      <c r="C97" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="D97" s="1" t="s">
+      <c r="D97" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="E97">
+      <c r="E97" s="1">
         <v>4</v>
       </c>
-      <c r="F97" t="s">
+      <c r="F97" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I97" t="s">
-        <v>402</v>
+      <c r="G97" s="1"/>
+      <c r="H97" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I97" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="98" spans="1:9">
-      <c r="A98" t="s">
+      <c r="A98" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B98">
+      <c r="B98" s="1">
         <v>2024</v>
       </c>
-      <c r="C98" t="s">
+      <c r="C98" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="D98" s="1" t="s">
+      <c r="D98" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="E98">
+      <c r="E98" s="1">
         <v>4</v>
       </c>
-      <c r="F98" t="s">
+      <c r="F98" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I98" t="s">
-        <v>402</v>
+      <c r="G98" s="1"/>
+      <c r="H98" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I98" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="99" spans="1:9">
-      <c r="A99" t="s">
+      <c r="A99" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B99">
+      <c r="B99" s="1">
         <v>1990</v>
       </c>
-      <c r="C99" t="s">
+      <c r="C99" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="D99" s="1" t="s">
+      <c r="D99" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="E99">
+      <c r="E99" s="1">
         <v>3</v>
       </c>
-      <c r="F99" t="s">
+      <c r="F99" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I99" t="s">
-        <v>402</v>
+      <c r="G99" s="1"/>
+      <c r="H99" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I99" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="100" spans="1:9">
-      <c r="A100" t="s">
+      <c r="A100" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B100">
+      <c r="B100" s="1">
         <v>1992</v>
       </c>
-      <c r="C100" t="s">
+      <c r="C100" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="D100" s="1" t="s">
+      <c r="D100" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="E100">
+      <c r="E100" s="1">
         <v>3</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F100" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I100" t="s">
-        <v>402</v>
+      <c r="G100" s="1"/>
+      <c r="H100" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I100" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="101" spans="1:9">
-      <c r="A101" t="s">
+      <c r="A101" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B101">
+      <c r="B101" s="1">
         <v>1992</v>
       </c>
-      <c r="C101" t="s">
+      <c r="C101" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="D101" s="1" t="s">
+      <c r="D101" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E101">
+      <c r="E101" s="1">
         <v>4</v>
       </c>
-      <c r="F101" t="s">
+      <c r="F101" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I101" t="s">
-        <v>402</v>
+      <c r="G101" s="1"/>
+      <c r="H101" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I101" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="102" spans="1:9">
-      <c r="A102" t="s">
+      <c r="A102" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B102">
+      <c r="B102" s="1">
         <v>1992</v>
       </c>
-      <c r="C102" t="s">
+      <c r="C102" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="D102" s="1" t="s">
+      <c r="D102" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="E102">
+      <c r="E102" s="1">
         <v>4</v>
       </c>
-      <c r="F102" t="s">
+      <c r="F102" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I102" t="s">
-        <v>402</v>
+      <c r="G102" s="1"/>
+      <c r="H102" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I102" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="103" spans="1:9">
-      <c r="A103" t="s">
+      <c r="A103" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B103">
+      <c r="B103" s="1">
         <v>1995</v>
       </c>
-      <c r="C103" t="s">
+      <c r="C103" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="D103" s="1" t="s">
+      <c r="D103" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="E103">
+      <c r="E103" s="1">
         <v>4</v>
       </c>
-      <c r="F103" t="s">
+      <c r="F103" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I103" t="s">
-        <v>402</v>
+      <c r="G103" s="1"/>
+      <c r="H103" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I103" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="104" spans="1:9">
-      <c r="A104" t="s">
+      <c r="A104" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="B104">
+      <c r="B104" s="1">
         <v>1997</v>
       </c>
-      <c r="C104" t="s">
+      <c r="C104" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="D104" s="1" t="s">
+      <c r="D104" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="E104">
+      <c r="E104" s="1">
         <v>3</v>
       </c>
-      <c r="F104" t="s">
+      <c r="F104" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I104" t="s">
-        <v>402</v>
+      <c r="G104" s="1"/>
+      <c r="H104" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I104" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="105" spans="1:9">
-      <c r="A105" t="s">
+      <c r="A105" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B105">
+      <c r="B105" s="1">
         <v>2002</v>
       </c>
-      <c r="C105" t="s">
+      <c r="C105" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D105" s="1" t="s">
+      <c r="D105" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="E105">
+      <c r="E105" s="1">
         <v>3</v>
       </c>
-      <c r="F105" t="s">
+      <c r="F105" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I105" t="s">
-        <v>402</v>
+      <c r="G105" s="1"/>
+      <c r="H105" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I105" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="106" spans="1:9">
-      <c r="A106" t="s">
+      <c r="A106" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B106">
+      <c r="B106" s="1">
         <v>2002</v>
       </c>
-      <c r="C106" t="s">
+      <c r="C106" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="D106" s="1" t="s">
+      <c r="D106" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="E106">
+      <c r="E106" s="1">
         <v>3</v>
       </c>
-      <c r="F106" t="s">
+      <c r="F106" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I106" t="s">
-        <v>402</v>
+      <c r="G106" s="1"/>
+      <c r="H106" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I106" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="107" spans="1:9">
-      <c r="A107" t="s">
+      <c r="A107" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B107">
+      <c r="B107" s="1">
         <v>2004</v>
       </c>
-      <c r="C107" t="s">
+      <c r="C107" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="D107" s="1" t="s">
+      <c r="D107" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="E107">
+      <c r="E107" s="1">
         <v>2</v>
       </c>
-      <c r="F107" t="s">
+      <c r="F107" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I107" t="s">
-        <v>402</v>
+      <c r="G107" s="1"/>
+      <c r="H107" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I107" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="108" spans="1:9">
-      <c r="A108" t="s">
+      <c r="A108" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B108">
+      <c r="B108" s="1">
         <v>2004</v>
       </c>
-      <c r="C108" t="s">
+      <c r="C108" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="D108" s="1" t="s">
+      <c r="D108" s="4" t="s">
         <v>376</v>
       </c>
-      <c r="E108">
+      <c r="E108" s="1">
         <v>3</v>
       </c>
-      <c r="F108" t="s">
+      <c r="F108" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I108" t="s">
-        <v>402</v>
+      <c r="G108" s="1"/>
+      <c r="H108" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I108" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="109" spans="1:9">
-      <c r="A109" t="s">
+      <c r="A109" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B109">
+      <c r="B109" s="1">
         <v>2004</v>
       </c>
-      <c r="C109" t="s">
+      <c r="C109" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="D109" s="1" t="s">
+      <c r="D109" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="E109">
+      <c r="E109" s="1">
         <v>3</v>
       </c>
-      <c r="F109" t="s">
+      <c r="F109" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I109" t="s">
-        <v>402</v>
+      <c r="G109" s="1"/>
+      <c r="H109" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I109" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="110" spans="1:9">
-      <c r="A110" t="s">
+      <c r="A110" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B110">
+      <c r="B110" s="1">
         <v>2005</v>
       </c>
-      <c r="C110" t="s">
+      <c r="C110" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="D110" s="1" t="s">
+      <c r="D110" s="4" t="s">
         <v>378</v>
       </c>
-      <c r="E110">
+      <c r="E110" s="1">
         <v>2</v>
       </c>
-      <c r="F110" t="s">
+      <c r="F110" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I110" t="s">
-        <v>402</v>
+      <c r="G110" s="1"/>
+      <c r="H110" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I110" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="111" spans="1:9">
-      <c r="A111" t="s">
+      <c r="A111" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B111">
+      <c r="B111" s="1">
         <v>2007</v>
       </c>
-      <c r="C111" t="s">
+      <c r="C111" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="D111" s="1" t="s">
+      <c r="D111" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="E111">
+      <c r="E111" s="1">
         <v>2</v>
       </c>
-      <c r="F111" t="s">
+      <c r="F111" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I111" t="s">
-        <v>402</v>
+      <c r="G111" s="1"/>
+      <c r="H111" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I111" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="112" spans="1:9">
-      <c r="A112" t="s">
+      <c r="A112" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B112">
+      <c r="B112" s="1">
         <v>2009</v>
       </c>
-      <c r="C112" t="s">
+      <c r="C112" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="D112" s="1" t="s">
+      <c r="D112" s="4" t="s">
         <v>380</v>
       </c>
-      <c r="E112">
+      <c r="E112" s="1">
         <v>2</v>
       </c>
-      <c r="F112" t="s">
+      <c r="F112" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I112" t="s">
-        <v>402</v>
+      <c r="G112" s="1"/>
+      <c r="H112" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I112" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="113" spans="1:9">
-      <c r="A113" t="s">
+      <c r="A113" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B113">
+      <c r="B113" s="1">
         <v>2009</v>
       </c>
-      <c r="C113" t="s">
+      <c r="C113" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="D113" s="1" t="s">
+      <c r="D113" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="E113">
+      <c r="E113" s="1">
         <v>2</v>
       </c>
-      <c r="F113" t="s">
+      <c r="F113" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I113" t="s">
-        <v>402</v>
+      <c r="G113" s="1"/>
+      <c r="H113" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I113" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="114" spans="1:9">
-      <c r="A114" t="s">
+      <c r="A114" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B114">
+      <c r="B114" s="1">
         <v>2010</v>
       </c>
-      <c r="C114" t="s">
+      <c r="C114" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="D114" s="1" t="s">
+      <c r="D114" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="E114">
+      <c r="E114" s="1">
         <v>3</v>
       </c>
-      <c r="F114" t="s">
+      <c r="F114" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I114" t="s">
-        <v>402</v>
+      <c r="G114" s="1"/>
+      <c r="H114" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I114" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="115" spans="1:9">
-      <c r="A115" t="s">
+      <c r="A115" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B115">
+      <c r="B115" s="2">
         <v>2011</v>
       </c>
-      <c r="C115" t="s">
+      <c r="C115" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="D115" s="1" t="s">
+      <c r="D115" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="E115">
+      <c r="E115" s="2">
         <v>2</v>
       </c>
-      <c r="F115" t="s">
+      <c r="F115" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I115" t="s">
-        <v>402</v>
+      <c r="G115" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H115" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I115" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="116" spans="1:9">
-      <c r="A116" t="s">
+      <c r="A116" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B116">
+      <c r="B116" s="2">
         <v>2011</v>
       </c>
-      <c r="C116" t="s">
+      <c r="C116" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="D116" s="1" t="s">
+      <c r="D116" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="E116">
+      <c r="E116" s="2">
         <v>2</v>
       </c>
-      <c r="F116" t="s">
+      <c r="F116" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="I116" t="s">
-        <v>402</v>
+      <c r="G116" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H116" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I116" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="117" spans="1:9">
-      <c r="A117" t="s">
+      <c r="A117" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B117">
+      <c r="B117" s="1">
         <v>2012</v>
       </c>
-      <c r="C117" t="s">
+      <c r="C117" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="D117" s="1" t="s">
+      <c r="D117" s="4" t="s">
         <v>385</v>
       </c>
-      <c r="E117">
+      <c r="E117" s="1">
         <v>2</v>
       </c>
-      <c r="F117" t="s">
+      <c r="F117" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I117" t="s">
-        <v>402</v>
+      <c r="G117" s="1"/>
+      <c r="H117" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I117" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="118" spans="1:9">
-      <c r="A118" t="s">
+      <c r="A118" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B118">
+      <c r="B118" s="1">
         <v>2012</v>
       </c>
-      <c r="C118" t="s">
+      <c r="C118" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="D118" s="1" t="s">
+      <c r="D118" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="E118">
+      <c r="E118" s="1">
         <v>3</v>
       </c>
-      <c r="F118" t="s">
+      <c r="F118" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I118" t="s">
-        <v>402</v>
+      <c r="G118" s="1"/>
+      <c r="H118" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I118" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="119" spans="1:9">
-      <c r="A119" t="s">
+      <c r="A119" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B119">
+      <c r="B119" s="1">
         <v>2013</v>
       </c>
-      <c r="C119" t="s">
+      <c r="C119" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="D119" s="1" t="s">
+      <c r="D119" s="4" t="s">
         <v>387</v>
       </c>
-      <c r="E119">
+      <c r="E119" s="1">
         <v>3</v>
       </c>
-      <c r="F119" t="s">
+      <c r="F119" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I119" t="s">
-        <v>402</v>
+      <c r="G119" s="1"/>
+      <c r="H119" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I119" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="120" spans="1:9">
-      <c r="A120" t="s">
+      <c r="A120" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B120">
+      <c r="B120" s="1">
         <v>2018</v>
       </c>
-      <c r="C120" t="s">
+      <c r="C120" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="D120" s="1" t="s">
+      <c r="D120" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="E120">
+      <c r="E120" s="1">
         <v>3</v>
       </c>
-      <c r="F120" t="s">
+      <c r="F120" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I120" t="s">
-        <v>402</v>
+      <c r="G120" s="1"/>
+      <c r="H120" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I120" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="121" spans="1:9">
-      <c r="A121" t="s">
+      <c r="A121" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B121">
+      <c r="B121" s="1">
         <v>2022</v>
       </c>
-      <c r="C121" t="s">
+      <c r="C121" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="D121" s="1" t="s">
+      <c r="D121" s="4" t="s">
         <v>389</v>
       </c>
-      <c r="E121">
+      <c r="E121" s="1">
         <v>2</v>
       </c>
-      <c r="F121" t="s">
+      <c r="F121" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I121" t="s">
-        <v>402</v>
+      <c r="G121" s="1"/>
+      <c r="H121" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I121" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="122" spans="1:9">
-      <c r="A122" t="s">
+      <c r="A122" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B122">
+      <c r="B122" s="1">
         <v>2023</v>
       </c>
-      <c r="C122" t="s">
+      <c r="C122" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="D122" s="1" t="s">
+      <c r="D122" s="4" t="s">
         <v>390</v>
       </c>
-      <c r="E122">
+      <c r="E122" s="1">
         <v>2</v>
       </c>
-      <c r="F122" t="s">
+      <c r="F122" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I122" t="s">
-        <v>402</v>
+      <c r="G122" s="1"/>
+      <c r="H122" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I122" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="123" spans="1:9">
-      <c r="A123" t="s">
+      <c r="A123" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B123">
+      <c r="B123" s="1">
         <v>2024</v>
       </c>
-      <c r="C123" t="s">
+      <c r="C123" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="D123" s="1" t="s">
+      <c r="D123" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="E123">
+      <c r="E123" s="1">
         <v>2</v>
       </c>
-      <c r="F123" t="s">
+      <c r="F123" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I123" t="s">
-        <v>402</v>
+      <c r="G123" s="1"/>
+      <c r="H123" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I123" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="124" spans="1:9">
-      <c r="A124" t="s">
+      <c r="A124" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B124">
+      <c r="B124" s="1">
         <v>2024</v>
       </c>
-      <c r="C124" t="s">
+      <c r="C124" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="D124" s="1" t="s">
+      <c r="D124" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="E124">
+      <c r="E124" s="1">
         <v>3</v>
       </c>
-      <c r="F124" t="s">
+      <c r="F124" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I124" t="s">
-        <v>402</v>
+      <c r="G124" s="1"/>
+      <c r="H124" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I124" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="125" spans="1:9">
-      <c r="A125" t="s">
+      <c r="A125" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B125">
+      <c r="B125" s="1">
         <v>2025</v>
       </c>
-      <c r="C125" t="s">
+      <c r="C125" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="D125" s="1" t="s">
+      <c r="D125" s="4" t="s">
         <v>393</v>
       </c>
-      <c r="E125">
+      <c r="E125" s="1">
         <v>2</v>
       </c>
-      <c r="F125" t="s">
+      <c r="F125" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I125" t="s">
-        <v>402</v>
+      <c r="G125" s="1"/>
+      <c r="H125" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I125" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
     <row r="126" spans="1:9">
-      <c r="A126" t="s">
+      <c r="A126" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B126">
+      <c r="B126" s="1">
         <v>1998</v>
       </c>
-      <c r="C126" t="s">
+      <c r="C126" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="D126" s="1" t="s">
+      <c r="D126" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="E126">
+      <c r="E126" s="1">
         <v>2</v>
       </c>
-      <c r="F126" t="s">
+      <c r="F126" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I126" t="s">
-        <v>402</v>
+      <c r="G126" s="1"/>
+      <c r="H126" s="5" t="s">
+        <v>1923</v>
+      </c>
+      <c r="I126" s="5" t="s">
+        <v>1924</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: lei-12067-29-outubro-2009-591929 - sem ementa e atualização planilha.
</commit_message>
<xml_diff>
--- a/avaliacao/Filipe/ouro_Filipe.xlsx
+++ b/avaliacao/Filipe/ouro_Filipe.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8879" uniqueCount="1930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8880" uniqueCount="1930">
   <si>
     <t>campo</t>
   </si>
@@ -9302,30 +9302,32 @@
       </c>
     </row>
     <row r="113" spans="1:9">
-      <c r="A113" s="1" t="s">
+      <c r="A113" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B113" s="1">
+      <c r="B113" s="2">
         <v>2009</v>
       </c>
-      <c r="C113" s="1" t="s">
+      <c r="C113" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D113" s="4" t="s">
+      <c r="D113" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E113" s="1">
+      <c r="E113" s="2">
         <v>2</v>
       </c>
-      <c r="F113" s="1" t="s">
+      <c r="F113" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="G113" s="1"/>
-      <c r="H113" s="5" t="s">
+      <c r="G113" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H113" s="2" t="s">
         <v>1923</v>
       </c>
-      <c r="I113" s="5" t="s">
-        <v>1924</v>
+      <c r="I113" s="2" t="s">
+        <v>1925</v>
       </c>
     </row>
     <row r="114" spans="1:9">

</xml_diff>